<commit_message>
Ship the three-sheet Week 2 worksheet, and put the deadline back on Tuesday
The Thursday hand-build now carries the two examples that used to live only on slides,
Anderson's four Finals free throws and Durant's 2010-11 game log, so students have
something to fill in rather than watch. The README gets a section per sheet.

The due date had reverted to Monday, September 7, which is Labor Day. A script rewrote
course-schedule.json from a stale read and took the objectives block with it.
</commit_message>
<xml_diff>
--- a/weeks/week02/data/hand-build-nfl-field-goals-worksheet.xlsx
+++ b/weeks/week02/data/hand-build-nfl-field-goals-worksheet.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="field goals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="free throws" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="game log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -59,7 +62,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -68,12 +71,29 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -435,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:T30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -454,6 +474,9 @@
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,12 +552,27 @@
       </c>
       <c r="P1" s="2" t="inlineStr">
         <is>
-          <t>Z vs league</t>
+          <t>Z score vs league</t>
         </is>
       </c>
       <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>Interval excludes league rate?</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>P(next two both made), multiplied</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>P(next two both made), BINOM.DIST</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>P(his makes or fewer, at the league rate)</t>
         </is>
       </c>
     </row>
@@ -573,8 +611,11 @@
       <c r="O2" s="5" t="n">
         <v>0.8421999999999999</v>
       </c>
-      <c r="P2" s="6" t="n"/>
+      <c r="P2" s="3" t="n"/>
       <c r="Q2" s="3" t="n"/>
+      <c r="R2" s="4" t="n"/>
+      <c r="S2" s="4" t="n"/>
+      <c r="T2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1253,13 +1294,1544 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Fill in every highlighted cell. Use cell references, not typed-in numbers, so the sheet still works if a row changes.</t>
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Fill in every highlighted cell. Each one turns from yellow to green when the answer in it is right, so a sheet with any yellow left in it is not finished. The check allows for rounding, so a value you rounded to three decimals still turns green. Use cell references, not typed-in numbers, so the sheet still works if a row changes. The two P(next two both made) cells ask for the same probability twice, once by multiplying the rate by itself and once with BINOM.DIST. They should agree to every decimal, and if they do not, your BINOM.DIST arguments are in the wrong order.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="H2">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(ISNUMBER(H2),ABS(H2-(COUNT($D$2:$D$28)))&lt;=MAX(0*ABS(COUNT($D$2:$D$28)),0))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>AND(ISNUMBER(I2),ABS(I2-(SUM($F$2:$F$28)))&lt;=MAX(0*ABS(SUM($F$2:$F$28)),0))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>AND(ISNUMBER(J2),ABS(J2-((SUM($F$2:$F$28)/COUNT($D$2:$D$28))))&lt;=MAX(0.02*ABS((SUM($F$2:$F$28)/COUNT($D$2:$D$28))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K2">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>AND(ISNUMBER(K2),ABS(K2-(SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28))))&lt;=MAX(0.02*ABS(SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2">
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>AND(ISNUMBER(L2),ABS(L2-(1.96*SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28))))&lt;=MAX(0.02*ABS(1.96*SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M2">
+    <cfRule type="expression" priority="6" dxfId="0">
+      <formula>AND(ISNUMBER(M2),ABS(M2-((SUM($F$2:$F$28)/COUNT($D$2:$D$28))-(1.96*SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))))&lt;=MAX(0.02*ABS((SUM($F$2:$F$28)/COUNT($D$2:$D$28))-(1.96*SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N2">
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>AND(ISNUMBER(N2),ABS(N2-((SUM($F$2:$F$28)/COUNT($D$2:$D$28))+(1.96*SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))))&lt;=MAX(0.02*ABS((SUM($F$2:$F$28)/COUNT($D$2:$D$28))+(1.96*SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P2">
+    <cfRule type="expression" priority="8" dxfId="0">
+      <formula>AND(ISNUMBER(P2),ABS(P2-(((SUM($F$2:$F$28)/COUNT($D$2:$D$28))-$O$2)/(SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))))&lt;=MAX(0.02*ABS(((SUM($F$2:$F$28)/COUNT($D$2:$D$28))-$O$2)/(SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q2">
+    <cfRule type="expression" priority="9" dxfId="0">
+      <formula>AND(Q2&lt;&gt;"",EXACT(LOWER(TRIM(Q2)),LOWER(IF(OR((SUM($F$2:$F$28)/COUNT($D$2:$D$28))+(1.96*SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))&lt;$O$2,(SUM($F$2:$F$28)/COUNT($D$2:$D$28))-(1.96*SQRT((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(1-(SUM($F$2:$F$28)/COUNT($D$2:$D$28)))/COUNT($D$2:$D$28)))&gt;$O$2),"yes","no"))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R2">
+    <cfRule type="expression" priority="10" dxfId="0">
+      <formula>AND(ISNUMBER(R2),ABS(R2-((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(SUM($F$2:$F$28)/COUNT($D$2:$D$28))))&lt;=MAX(0.02*ABS((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(SUM($F$2:$F$28)/COUNT($D$2:$D$28))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S2">
+    <cfRule type="expression" priority="11" dxfId="0">
+      <formula>AND(ISNUMBER(S2),ABS(S2-((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(SUM($F$2:$F$28)/COUNT($D$2:$D$28))))&lt;=MAX(0.02*ABS((SUM($F$2:$F$28)/COUNT($D$2:$D$28))*(SUM($F$2:$F$28)/COUNT($D$2:$D$28))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T2">
+    <cfRule type="expression" priority="12" dxfId="0">
+      <formula>AND(ISNUMBER(T2),ABS(T2-(_xlfn.BINOM.DIST(SUM($F$2:$F$28),COUNT($D$2:$D$28),$O$2,TRUE)))&lt;=MAX(0.02*ABS(_xlfn.BINOM.DIST(SUM($F$2:$F$28),COUNT($D$2:$D$28),$O$2,TRUE)),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Nick Anderson</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Free throw rate</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Season</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1994-95</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>P(miss on one attempt)</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Free throws made</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>143</v>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>P(misses all four), rate multiplied</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Free throws attempted</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>203</v>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>P(misses all four), BINOM.DIST</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Attempts in the Finals sequence</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>P(makes at least one of the four)</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Work the chance he misses all four twice, once by multiplying the miss rate by itself and once with BINOM.DIST, and check that the two agree to every decimal. If they do not, the arguments to BINOM.DIST are in the wrong order. Both routes assume the four attempts are independent of each other and that his season rate is the right rate for those four attempts. Be ready to say in class which of those two assumptions you trust less.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E1">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(ISNUMBER(E1),ABS(E1-(($B$3/$B$4)))&lt;=MAX(0.02*ABS(($B$3/$B$4)),0.002))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>AND(ISNUMBER(E2),ABS(E2-((1-($B$3/$B$4))))&lt;=MAX(0.02*ABS((1-($B$3/$B$4))),0.002))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E3">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>AND(ISNUMBER(E3),ABS(E3-((1-($B$3/$B$4))^$B$5))&lt;=MAX(0.02*ABS((1-($B$3/$B$4))^$B$5),0.0002))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E4">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>AND(ISNUMBER(E4),ABS(E4-((1-($B$3/$B$4))^$B$5))&lt;=MAX(0.02*ABS((1-($B$3/$B$4))^$B$5),0.0002))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5">
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>AND(ISNUMBER(E5),ABS(E5-((1-(1-($B$3/$B$4))^$B$5)))&lt;=MAX(0.02*ABS((1-(1-($B$3/$B$4))^$B$5)),0.002))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I79"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PTS</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>TRB</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>AST</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Statistic</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Rebounds</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Assists</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="n"/>
+      <c r="H2" s="9" t="n"/>
+      <c r="I2" s="9" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>28</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Standard deviation</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Standard error</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>28</v>
+      </c>
+      <c r="C6" t="n">
+        <v>11</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Relative spread</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>34</v>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>95% interval low</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>31</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>95% interval high</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>34</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Standard errors between his average and 30 points a game</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>23</v>
+      </c>
+      <c r="C10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>30</v>
+      </c>
+      <c r="C11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Relative spread is the standard deviation divided by the average, which is the coefficient of variation from Week 1. It puts three statistics on three different scales in one column. The same 78 games produced all three columns, so anything that differs between them is the spread of the statistic and nothing else. Use COUNT, AVERAGE, STDEV.S and SQRT, and build every cell from cell references.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>24</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>28</v>
+      </c>
+      <c r="C13" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>32</v>
+      </c>
+      <c r="C14" t="n">
+        <v>11</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>25</v>
+      </c>
+      <c r="C15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>18</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>26</v>
+      </c>
+      <c r="C17" t="n">
+        <v>11</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>28</v>
+      </c>
+      <c r="C18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>29</v>
+      </c>
+      <c r="C19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>30</v>
+      </c>
+      <c r="C20" t="n">
+        <v>11</v>
+      </c>
+      <c r="D20" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>25</v>
+      </c>
+      <c r="C21" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>25</v>
+      </c>
+      <c r="C22" t="n">
+        <v>7</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>32</v>
+      </c>
+      <c r="C23" t="n">
+        <v>7</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>24</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>28</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>32</v>
+      </c>
+      <c r="C26" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="n">
+        <v>7</v>
+      </c>
+      <c r="D27" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>44</v>
+      </c>
+      <c r="C28" t="n">
+        <v>7</v>
+      </c>
+      <c r="D28" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>27</v>
+      </c>
+      <c r="C30" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>33</v>
+      </c>
+      <c r="C31" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>16</v>
+      </c>
+      <c r="C32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>28</v>
+      </c>
+      <c r="C33" t="n">
+        <v>9</v>
+      </c>
+      <c r="D33" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>28</v>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>40</v>
+      </c>
+      <c r="C35" t="n">
+        <v>8</v>
+      </c>
+      <c r="D35" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>30</v>
+      </c>
+      <c r="C36" t="n">
+        <v>6</v>
+      </c>
+      <c r="D36" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="n">
+        <v>4</v>
+      </c>
+      <c r="D37" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>24</v>
+      </c>
+      <c r="C38" t="n">
+        <v>8</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>22</v>
+      </c>
+      <c r="C39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>30</v>
+      </c>
+      <c r="C40" t="n">
+        <v>12</v>
+      </c>
+      <c r="D40" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>22</v>
+      </c>
+      <c r="C41" t="n">
+        <v>8</v>
+      </c>
+      <c r="D41" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>47</v>
+      </c>
+      <c r="C42" t="n">
+        <v>18</v>
+      </c>
+      <c r="D42" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>40</v>
+      </c>
+      <c r="C43" t="n">
+        <v>7</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="n">
+        <v>33</v>
+      </c>
+      <c r="C44" t="n">
+        <v>10</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>43</v>
+      </c>
+      <c r="C45" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>24</v>
+      </c>
+      <c r="C46" t="n">
+        <v>11</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>21</v>
+      </c>
+      <c r="C47" t="n">
+        <v>12</v>
+      </c>
+      <c r="D47" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="n">
+        <v>31</v>
+      </c>
+      <c r="C48" t="n">
+        <v>10</v>
+      </c>
+      <c r="D48" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="n">
+        <v>35</v>
+      </c>
+      <c r="C49" t="n">
+        <v>6</v>
+      </c>
+      <c r="D49" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="n">
+        <v>29</v>
+      </c>
+      <c r="C50" t="n">
+        <v>5</v>
+      </c>
+      <c r="D50" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="n">
+        <v>17</v>
+      </c>
+      <c r="C51" t="n">
+        <v>7</v>
+      </c>
+      <c r="D51" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="n">
+        <v>21</v>
+      </c>
+      <c r="C52" t="n">
+        <v>8</v>
+      </c>
+      <c r="D52" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="n">
+        <v>30</v>
+      </c>
+      <c r="C53" t="n">
+        <v>9</v>
+      </c>
+      <c r="D53" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="n">
+        <v>23</v>
+      </c>
+      <c r="C54" t="n">
+        <v>16</v>
+      </c>
+      <c r="D54" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="n">
+        <v>21</v>
+      </c>
+      <c r="C55" t="n">
+        <v>4</v>
+      </c>
+      <c r="D55" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="n">
+        <v>21</v>
+      </c>
+      <c r="C56" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="n">
+        <v>29</v>
+      </c>
+      <c r="C57" t="n">
+        <v>8</v>
+      </c>
+      <c r="D57" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="n">
+        <v>18</v>
+      </c>
+      <c r="C58" t="n">
+        <v>8</v>
+      </c>
+      <c r="D58" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="n">
+        <v>23</v>
+      </c>
+      <c r="C59" t="n">
+        <v>6</v>
+      </c>
+      <c r="D59" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="n">
+        <v>34</v>
+      </c>
+      <c r="C60" t="n">
+        <v>16</v>
+      </c>
+      <c r="D60" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="n">
+        <v>24</v>
+      </c>
+      <c r="C61" t="n">
+        <v>9</v>
+      </c>
+      <c r="D61" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="n">
+        <v>19</v>
+      </c>
+      <c r="C62" t="n">
+        <v>3</v>
+      </c>
+      <c r="D62" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="n">
+        <v>32</v>
+      </c>
+      <c r="C63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D63" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="n">
+        <v>29</v>
+      </c>
+      <c r="C64" t="n">
+        <v>7</v>
+      </c>
+      <c r="D64" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="n">
+        <v>25</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="n">
+        <v>20</v>
+      </c>
+      <c r="C66" t="n">
+        <v>5</v>
+      </c>
+      <c r="D66" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="n">
+        <v>29</v>
+      </c>
+      <c r="C67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="n">
+        <v>23</v>
+      </c>
+      <c r="C68" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="n">
+        <v>21</v>
+      </c>
+      <c r="C69" t="n">
+        <v>3</v>
+      </c>
+      <c r="D69" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="n">
+        <v>39</v>
+      </c>
+      <c r="C70" t="n">
+        <v>6</v>
+      </c>
+      <c r="D70" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="n">
+        <v>22</v>
+      </c>
+      <c r="C71" t="n">
+        <v>4</v>
+      </c>
+      <c r="D71" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="n">
+        <v>25</v>
+      </c>
+      <c r="C72" t="n">
+        <v>11</v>
+      </c>
+      <c r="D72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="n">
+        <v>23</v>
+      </c>
+      <c r="C73" t="n">
+        <v>6</v>
+      </c>
+      <c r="D73" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="n">
+        <v>32</v>
+      </c>
+      <c r="C74" t="n">
+        <v>9</v>
+      </c>
+      <c r="D74" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="n">
+        <v>29</v>
+      </c>
+      <c r="C75" t="n">
+        <v>7</v>
+      </c>
+      <c r="D75" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="n">
+        <v>28</v>
+      </c>
+      <c r="C76" t="n">
+        <v>7</v>
+      </c>
+      <c r="D76" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="n">
+        <v>31</v>
+      </c>
+      <c r="C77" t="n">
+        <v>4</v>
+      </c>
+      <c r="D77" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="n">
+        <v>32</v>
+      </c>
+      <c r="C78" t="n">
+        <v>8</v>
+      </c>
+      <c r="D78" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="n">
+        <v>14</v>
+      </c>
+      <c r="C79" t="n">
+        <v>6</v>
+      </c>
+      <c r="D79" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="G2">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(ISNUMBER(G2),ABS(G2-(COUNT($B$2:$B$79)))&lt;=MAX(0*ABS(COUNT($B$2:$B$79)),0))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G3">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>AND(ISNUMBER(G3),ABS(G3-(AVERAGE($B$2:$B$79)))&lt;=MAX(0.02*ABS(AVERAGE($B$2:$B$79)),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>AND(ISNUMBER(G4),ABS(G4-(_xlfn.STDEV.S($B$2:$B$79)))&lt;=MAX(0.02*ABS(_xlfn.STDEV.S($B$2:$B$79)),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>AND(ISNUMBER(G5),ABS(G5-((_xlfn.STDEV.S($B$2:$B$79)/SQRT(COUNT($B$2:$B$79)))))&lt;=MAX(0.02*ABS((_xlfn.STDEV.S($B$2:$B$79)/SQRT(COUNT($B$2:$B$79)))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G6">
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>AND(ISNUMBER(G6),ABS(G6-((_xlfn.STDEV.S($B$2:$B$79)/AVERAGE($B$2:$B$79))))&lt;=MAX(0.02*ABS((_xlfn.STDEV.S($B$2:$B$79)/AVERAGE($B$2:$B$79))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7">
+    <cfRule type="expression" priority="6" dxfId="0">
+      <formula>AND(ISNUMBER(G7),ABS(G7-((AVERAGE($B$2:$B$79)-1.96*(_xlfn.STDEV.S($B$2:$B$79)/SQRT(COUNT($B$2:$B$79))))))&lt;=MAX(0.02*ABS((AVERAGE($B$2:$B$79)-1.96*(_xlfn.STDEV.S($B$2:$B$79)/SQRT(COUNT($B$2:$B$79))))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8">
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>AND(ISNUMBER(G8),ABS(G8-((AVERAGE($B$2:$B$79)+1.96*(_xlfn.STDEV.S($B$2:$B$79)/SQRT(COUNT($B$2:$B$79))))))&lt;=MAX(0.02*ABS((AVERAGE($B$2:$B$79)+1.96*(_xlfn.STDEV.S($B$2:$B$79)/SQRT(COUNT($B$2:$B$79))))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2">
+    <cfRule type="expression" priority="8" dxfId="0">
+      <formula>AND(ISNUMBER(H2),ABS(H2-(COUNT($C$2:$C$79)))&lt;=MAX(0*ABS(COUNT($C$2:$C$79)),0))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" priority="9" dxfId="0">
+      <formula>AND(ISNUMBER(H3),ABS(H3-(AVERAGE($C$2:$C$79)))&lt;=MAX(0.02*ABS(AVERAGE($C$2:$C$79)),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="expression" priority="10" dxfId="0">
+      <formula>AND(ISNUMBER(H4),ABS(H4-(_xlfn.STDEV.S($C$2:$C$79)))&lt;=MAX(0.02*ABS(_xlfn.STDEV.S($C$2:$C$79)),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H5">
+    <cfRule type="expression" priority="11" dxfId="0">
+      <formula>AND(ISNUMBER(H5),ABS(H5-((_xlfn.STDEV.S($C$2:$C$79)/SQRT(COUNT($C$2:$C$79)))))&lt;=MAX(0.02*ABS((_xlfn.STDEV.S($C$2:$C$79)/SQRT(COUNT($C$2:$C$79)))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H6">
+    <cfRule type="expression" priority="12" dxfId="0">
+      <formula>AND(ISNUMBER(H6),ABS(H6-((_xlfn.STDEV.S($C$2:$C$79)/AVERAGE($C$2:$C$79))))&lt;=MAX(0.02*ABS((_xlfn.STDEV.S($C$2:$C$79)/AVERAGE($C$2:$C$79))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H7">
+    <cfRule type="expression" priority="13" dxfId="0">
+      <formula>AND(ISNUMBER(H7),ABS(H7-((AVERAGE($C$2:$C$79)-1.96*(_xlfn.STDEV.S($C$2:$C$79)/SQRT(COUNT($C$2:$C$79))))))&lt;=MAX(0.02*ABS((AVERAGE($C$2:$C$79)-1.96*(_xlfn.STDEV.S($C$2:$C$79)/SQRT(COUNT($C$2:$C$79))))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H8">
+    <cfRule type="expression" priority="14" dxfId="0">
+      <formula>AND(ISNUMBER(H8),ABS(H8-((AVERAGE($C$2:$C$79)+1.96*(_xlfn.STDEV.S($C$2:$C$79)/SQRT(COUNT($C$2:$C$79))))))&lt;=MAX(0.02*ABS((AVERAGE($C$2:$C$79)+1.96*(_xlfn.STDEV.S($C$2:$C$79)/SQRT(COUNT($C$2:$C$79))))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2">
+    <cfRule type="expression" priority="15" dxfId="0">
+      <formula>AND(ISNUMBER(I2),ABS(I2-(COUNT($D$2:$D$79)))&lt;=MAX(0*ABS(COUNT($D$2:$D$79)),0))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3">
+    <cfRule type="expression" priority="16" dxfId="0">
+      <formula>AND(ISNUMBER(I3),ABS(I3-(AVERAGE($D$2:$D$79)))&lt;=MAX(0.02*ABS(AVERAGE($D$2:$D$79)),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I4">
+    <cfRule type="expression" priority="17" dxfId="0">
+      <formula>AND(ISNUMBER(I4),ABS(I4-(_xlfn.STDEV.S($D$2:$D$79)))&lt;=MAX(0.02*ABS(_xlfn.STDEV.S($D$2:$D$79)),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5">
+    <cfRule type="expression" priority="18" dxfId="0">
+      <formula>AND(ISNUMBER(I5),ABS(I5-((_xlfn.STDEV.S($D$2:$D$79)/SQRT(COUNT($D$2:$D$79)))))&lt;=MAX(0.02*ABS((_xlfn.STDEV.S($D$2:$D$79)/SQRT(COUNT($D$2:$D$79)))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6">
+    <cfRule type="expression" priority="19" dxfId="0">
+      <formula>AND(ISNUMBER(I6),ABS(I6-((_xlfn.STDEV.S($D$2:$D$79)/AVERAGE($D$2:$D$79))))&lt;=MAX(0.02*ABS((_xlfn.STDEV.S($D$2:$D$79)/AVERAGE($D$2:$D$79))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I7">
+    <cfRule type="expression" priority="20" dxfId="0">
+      <formula>AND(ISNUMBER(I7),ABS(I7-((AVERAGE($D$2:$D$79)-1.96*(_xlfn.STDEV.S($D$2:$D$79)/SQRT(COUNT($D$2:$D$79))))))&lt;=MAX(0.02*ABS((AVERAGE($D$2:$D$79)-1.96*(_xlfn.STDEV.S($D$2:$D$79)/SQRT(COUNT($D$2:$D$79))))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I8">
+    <cfRule type="expression" priority="21" dxfId="0">
+      <formula>AND(ISNUMBER(I8),ABS(I8-((AVERAGE($D$2:$D$79)+1.96*(_xlfn.STDEV.S($D$2:$D$79)/SQRT(COUNT($D$2:$D$79))))))&lt;=MAX(0.02*ABS((AVERAGE($D$2:$D$79)+1.96*(_xlfn.STDEV.S($D$2:$D$79)/SQRT(COUNT($D$2:$D$79))))),0.005))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="expression" priority="22" dxfId="0">
+      <formula>AND(ISNUMBER(G9),ABS(G9-(((30-AVERAGE($B$2:$B$79))/(_xlfn.STDEV.S($B$2:$B$79)/SQRT(COUNT($B$2:$B$79))))))&lt;=MAX(0.02*ABS(((30-AVERAGE($B$2:$B$79))/(_xlfn.STDEV.S($B$2:$B$79)/SQRT(COUNT($B$2:$B$79))))),0.05))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>